<commit_message>
Keep tests off the production database; selective JSON import
backend/.env now points at the real Supabase database, so an autouse test
fixture makes any test that reaches for it fail instead of writing there.

- migrate_json_documents gains --only, used to import just the owner's two
  real documents out of the old JSON store (the rest were test leftovers).
- Docs: the backend connects as a least-privilege role (data read/write, no
  schema changes); schema changes are applied separately.
- Tracker: Phases 3, 5 and 6 verified live in the signed-in UI on Supabase.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/saas-transformation-tracker.xlsx
+++ b/saas-transformation-tracker.xlsx
@@ -761,7 +761,7 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Postgres host: Supabase (managed Postgres 17.6), project smartdoc-formatter (ref edmmjmsynjziahwtjuke, eu-central-1 Frankfurt, Free plan, $0/month), created through the Supabase MCP connector after the local Windows Postgres install hit an unresolvable auth problem. Schema applied from Alembic's own offline-rendered PostgreSQL SQL (alembic upgrade --sql), one Supabase migration per Alembic revision, so alembic_version in the DB equals the code head (e7958c683f5b) and a later `alembic upgrade head` from the backend is a no-op. 3 revisions: 361677e33e9c initial schema; 4cbc55236361 enables RLS on every table -- Supabase exposes public tables over its REST/GraphQL Data API and grants the public anon role SELECT by default (confirmed live: has_table_privilege('anon', ...) = true), so without it every document would have been readable/writable by anyone holding the public key; the backend connects as owner `postgres` (BYPASSRLS) and is unaffected; guarded by test_every_table_gets_rls_enabled_on_postgres, which renders the whole chain as Postgres SQL offline and fails if any CREATE TABLE lacks a matching ENABLE RLS; e7958c683f5b indexes the 8 FK columns Supabase's performance advisor flagged (free now, expensive on populated tables later). Verified live on Supabase: 15 tables all RLS-enabled, 22 FKs, 3 unique constraints, 43 indexes; JSONB with Cyrillic round-trips and is path-queryable; FK violation rejected (23503); ON DELETE CASCADE removes a workspace's documents+versions; the REST API with the public key returns [] on read and 401/42501 on write even with rows present. Advisors: security = only INFO 'RLS enabled, no policy' (intentional default-deny), performance = only INFO 'unused index' (empty DB, never queried). Smoke-test rows cleaned up. Settings.database_url normalizes a pasted Supabase URI (postgres:// or postgresql:// -&gt; postgresql+asyncpg://, adds ssl=require for non-loopback hosts unless an explicit ssl param is given) -- 7 tests in test_config.py; engine uses pool_pre_ping (Supavisor drops idle connections). scripts/verify_database.py: one-command end-to-end check through the app's own engine (server version, DB head vs code head, DocumentRepository round-trip, always rolled back) -- dry-run verified against SQLite. Also found and fixed a gap in my own earlier tests: test_document_repository.py fetched through the session identity map, so it never actually read the JSON column back -- now expunges first. STILL NEEDED: the backend's own connection (asyncpg over the session pooler) -- waiting on Boril to reset the DB password and put the Session pooler URI in backend/.env, then run scripts.verify_database. Phase 15 follow-up: ssl=require encrypts but doesn't verify the server certificate; verify-full needs Supabase's CA cert.</t>
+          <t>Postgres host: Supabase (managed Postgres 17.6), project smartdoc-formatter (ref edmmjmsynjziahwtjuke, eu-central-1 Frankfurt, Free plan, $0/month), created through the Supabase MCP connector after the local Windows Postgres install hit an unresolvable auth problem. Schema applied from Alembic's own offline-rendered PostgreSQL SQL (alembic upgrade --sql), one Supabase migration per Alembic revision, so alembic_version in the DB equals the code head (e7958c683f5b) and a later `alembic upgrade head` from the backend is a no-op. 3 revisions: 361677e33e9c initial schema; 4cbc55236361 enables RLS on every table -- Supabase exposes public tables over its REST/GraphQL Data API and grants the public anon role SELECT by default (confirmed live: has_table_privilege('anon', ...) = true), so without it every document would have been readable/writable by anyone holding the public key; the backend connects as owner `postgres` (BYPASSRLS) and is unaffected; guarded by test_every_table_gets_rls_enabled_on_postgres, which renders the whole chain as Postgres SQL offline and fails if any CREATE TABLE lacks a matching ENABLE RLS; e7958c683f5b indexes the 8 FK columns Supabase's performance advisor flagged (free now, expensive on populated tables later). Verified live on Supabase: 15 tables all RLS-enabled, 22 FKs, 3 unique constraints, 43 indexes; JSONB with Cyrillic round-trips and is path-queryable; FK violation rejected (23503); ON DELETE CASCADE removes a workspace's documents+versions; the REST API with the public key returns [] on read and 401/42501 on write even with rows present. Advisors: security = only INFO 'RLS enabled, no policy' (intentional default-deny), performance = only INFO 'unused index' (empty DB, never queried). Smoke-test rows cleaned up. Settings.database_url normalizes a pasted Supabase URI (postgres:// or postgresql:// -&gt; postgresql+asyncpg://, adds ssl=require for non-loopback hosts unless an explicit ssl param is given) -- 7 tests in test_config.py; engine uses pool_pre_ping (Supavisor drops idle connections). scripts/verify_database.py: one-command end-to-end check through the app's own engine (server version, DB head vs code head, DocumentRepository round-trip, always rolled back) -- dry-run verified against SQLite. Also found and fixed a gap in my own earlier tests: test_document_repository.py fetched through the session identity map, so it never actually read the JSON column back -- now expunges first. Backend connection verified end to end (2026-09-24): the app logs in as a dedicated role smartdoc_app, created through the connector with a pre-hashed SCRAM secret (plaintext only in the gitignored backend/.env). It has data read/write on the public tables (read-only on alembic_version), bypasses RLS, and has no DDL rights and no access to Supabase's other schemas -- least privilege, instead of connecting as postgres. scripts.verify_database through the app's own engine: asyncpg over the session pooler with TLS, schema head matches code, repository round trip OK (rolled back). Phase 15 follow-up: ssl=require encrypts but doesn't verify the server certificate; verify-full needs Supabase's CA cert.</t>
         </is>
       </c>
     </row>
@@ -967,7 +967,7 @@
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>app/api/auth.py: POST /register (user + personal workspace + owner membership, signs in), /login, /logout (revokes the session server-side), GET /me. Frontend: /login and /register pages (shared AuthForm), a ?next= return path validated against open redirects, and an account menu with sign-out in the header. 16 API + 2 service tests. Live: signed-out visitors get sent to login from both server-rendered pages and client-side calls, and an off-site ?next= is neutralized; register/me/login/cross-user access verified with curl against the running server. The browser check of the signed-in screens is still pending: I don't type passwords into the browser, so it waits for Boril's own first sign-in.</t>
+          <t>app/api/auth.py: POST /register (user + personal workspace + owner membership, signs in), /login, /logout (revokes the session server-side), GET /me. Frontend: /login and /register pages (shared AuthForm), a ?next= return path validated against open redirects, and an account menu with sign-out in the header. 16 API + 2 service tests. Live: signed-out visitors get sent to login from both server-rendered pages and client-side calls, and an off-site ?next= is neutralized; register/me/login/cross-user access verified with curl against the running server. Verified live on Supabase after Boril registered in the browser pane himself (2026-09-24): account stored with an argon2id hash, owner of his Personal workspace; the editor opens his documents server-side through the forwarded cookie; the header shows his name with sign-out.</t>
         </is>
       </c>
     </row>
@@ -1079,7 +1079,7 @@
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>Kept exactly as it was: the Toolbar's undo/redo is ProseMirror's client-side text history and never calls the server; 'Undo formatting'/'Redo formatting' is the server history above. One behavior to know: autosaved typing is also a server step (merged per minute), so 'Undo formatting' right after typing undoes that typing burst first -- nothing is lost, redo brings it back. Not yet re-verified in the browser (needs Boril's sign-in).</t>
+          <t>Kept exactly as it was: the Toolbar's undo/redo is ProseMirror's client-side text history and never calls the server; 'Undo formatting'/'Redo formatting' is the server history above. One behavior to know: autosaved typing is also a server step (merged per minute), so 'Undo formatting' right after typing undoes that typing burst first -- nothing is lost, redo brings it back. Verified live in the signed-in UI: 'Undo formatting' reverted a rename made from another tab, through the revision-checked write queue.</t>
         </is>
       </c>
     </row>
@@ -1097,7 +1097,7 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>documents.revision is SQLAlchemy's version_id_col: every write bumps it, and an UPDATE only succeeds while it still matches what the request loaded. Document.revision rides on every API response; the client sends it back as If-Match (plain, quoted or W/ form), a mismatch answers 412 {currentRevision} and writes nothing. Two requests racing between load and commit are caught by the row version (StaleDataError -&gt; same 412); a test reproduces that exact interleaving. Frontend: writes are queued one at a time per document and each response's revision is recorded before the next write starts, so a tab never conflicts with itself; a 412 shows a reload banner in the editor. 13 new tests. Live: If-Match 1 -&gt; 200 (rev 2), If-Match 2 -&gt; 200 (rev 3), stale If-Match 2 -&gt; 412 {currentRevision: 3}. The banner itself still needs a signed-in browser check.</t>
+          <t>documents.revision is SQLAlchemy's version_id_col: every write bumps it, and an UPDATE only succeeds while it still matches what the request loaded. Document.revision rides on every API response; the client sends it back as If-Match (plain, quoted or W/ form), a mismatch answers 412 {currentRevision} and writes nothing. Two requests racing between load and commit are caught by the row version (StaleDataError -&gt; same 412); a test reproduces that exact interleaving. Frontend: writes are queued one at a time per document and each response's revision is recorded before the next write starts, so a tab never conflicts with itself; a 412 shows a reload banner in the editor. 13 new tests. Live: If-Match 1 -&gt; 200 (rev 2), If-Match 2 -&gt; 200 (rev 3), stale If-Match 2 -&gt; 412 {currentRevision: 3}. Verified live in the signed-in UI: after another tab renamed the document, typing here autosaved with the stale revision -&gt; PUT 412 -&gt; amber banner -&gt; Reload showed the other tab's version; nothing was overwritten.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Keep what the editor can't show and put it back on export to Word
The preservation layer (корекции.docx §11). Equations (as the original OMML),
Word fields, bookmarks, links to bookmarks and comments are no longer
reduced to text or left out on import. The reader marks where each starts
and ends, the importer keeps them with their paragraph in
preservedAttributes["ooxml"], and the DOCX export puts each back wherever
its text still is: the real equation, the field with its last result, the
bookmark, the internal link, the comment with its author and date. Edited
text drops the piece, never the text. Everything is validated on export,
since it comes back from the browser on each autosave. Inside lists,
tables and footnotes the pieces stay text, with a note.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/saas-transformation-tracker.xlsx
+++ b/saas-transformation-tracker.xlsx
@@ -1320,12 +1320,12 @@
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>☑</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>Partly done. The importer reads the raw XML wherever python-docx stops (docx_inline.py, docx_styles.py): fields incl. HYPERLINK, content controls, OMML equations, footnote/endnote references, tracked changes, text boxes, VML, symbol-font characters, theme fonts, numbering. Still open: nothing is kept as opaque OOXML in Element.preservedAttributes yet (no producer). What can't be represented is reported in unsupportedFeatures instead, including bookmarks (added now: they used to disappear without a note).</t>
+          <t>Done. The importer reads the raw XML wherever python-docx stops (docx_inline.py, docx_styles.py): fields incl. HYPERLINK, content controls, OMML, notes, tracked changes, text boxes, VML, symbol fonts, theme fonts, numbering, comments (python-docx 1.2). Preservation layer (§11): equations (the original OMML), Word fields (instruction + last result), bookmarks (except _GoBack), links to bookmarks and comments (author, initials, date, text) leave start/end marker runs that survive the importer's run transformations; for text paragraphs they become Element.preservedAttributes["ooxml"] entries with their span and text. The DOCX export finds each one's text in the paragraph as it is now (at the old place, else the nearest occurrence) and puts it back: OMML in place of the linear text, fldChar begin/instr/separate/end around the result, bookmarkStart/End, w:hyperlink w:anchor, add_comment with the original date. Changed text drops the piece, never the text. Everything is validated on export (it comes back from the browser on each autosave). Inside lists/tables/footnotes/code: kept only as text, with a note. A table of contents stays plain text. tests/test_docx_preservation.py (9); all paths export schema-valid (OOXML validator), and Boril's stress document now keeps its 'TestSection' bookmark.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tick the SaaS transformation tracker's phases 11-18
The tracker updates written while Excel had the file open, applied once it
was closed: 90 of 91 tasks done; only the Stripe plans row stays open.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/saas-transformation-tracker.xlsx
+++ b/saas-transformation-tracker.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D83"/>
+  <dimension ref="A1:D92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1472,10 +1472,14 @@
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="D54" s="3" t="inlineStr"/>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>app/worker.py: the arq worker (run_job; up to 3 tries, 10 minutes each; the job-file sweep hourly and the unused-image sweep daily as cron jobs). app/jobs/queue.py picks where jobs run from JOB_BACKEND: background (in the API process, the development default; a restart fails what was running), arq (Redis at REDIS_URL, run `arq app.worker.WorkerSettings`), eager (tests). The job id doubles as arq's, so a job is never queued twice, and a job that can't be handed over fails at once with a 503 instead of waiting forever. Not yet run against a real Redis (none on this machine; Phase 17's compose file brings one): the arq path is tested with a fake pool and by calling the worker's function directly.</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n"/>
@@ -1486,10 +1490,14 @@
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="D55" s="3" t="inlineStr"/>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>Pasted-text import (AI structure analysis for plain prose), formatting with instructions (AI instruction extraction) and Format by Example (AI heading labels) run as jobs: POST /api/jobs/import-text, /format and /extract-reference answer 202 at once, after checking what can be checked up front (access, file type, size). The app uses only these; the earlier synchronous endpoints stay for API clients and tests. A finished job keeps no copy of the pasted text or instructions.</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n"/>
@@ -1500,10 +1508,14 @@
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="D56" s="3" t="inlineStr"/>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>File import (DOCX/PDF/TXT parsing) and DOCX/PDF export are jobs too (/import-file, /export). An upload waits in storage at jobs/{id}/input until its job has run; an export's file stays at jobs/{id}/output for JOB_FILE_TTL_HOURS (24), downloaded from GET /api/jobs/{id}/file, and goes at once when its document is deleted. app/jobs/files.py: the hourly sweep expires old export files (and any whose document is gone) and removes job rows after JOB_RETENTION_DAYS (7). Migration 5f5c3a367f6f (processing_jobs gets creator, stage, progress, payload, input, result, attempts; the unused export_jobs table is dropped) applied to Supabase after checking both tables were empty.</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n"/>
@@ -1514,76 +1526,96 @@
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="D57" s="3" t="inlineStr"/>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>Stage (queued, uploading, parsing, analyzing, formatting, rendering, finalizing, then complete or failed) and progress are written and committed only as real steps finish; services/api.ts waitForJob polls every 300 ms, slowing to 1.5 s. The new-document wizard lists each job's steps; the formatting panels, the conflict dialog, Format by Example (editor, wizard, library) and the export menu show a progress bar where the action was started (JobProgressBar). The editor is read-only while formatting runs, and the formatting job holds the document's write queue, so autosave follows with the new revision instead of a 412; export saves pending typing first. Also fixed: the quick AI bar's first submit sent the previous instructions. tests/test_jobs.py (22); checked live against Supabase (paste and DOCX import, formatting, a resolved conflict, exports, Format by Example in all three places, a broken file's error).</t>
+        </is>
+      </c>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="inlineStr">
+      <c r="A58" s="2" t="n"/>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>Unused-image sweep (the asset deletion Phase 4 deferred to a sweep)</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>services/asset_cleanup.py, daily (worker cron, or the API with in-process jobs): an image goes once no document of its workspace refers to it, in its content or its undo history, and it is over a day old; the row is committed away before the file is deleted. Deleting a document leaves its images to the sweep, since an image copied into another document of the workspace still points at them. Dry-run against Supabase before enabling it: only the 6 images of deleted test documents qualify. Not covered: a file whose row was never committed (storage can't be listed yet). tests/test_asset_cleanup.py.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
         <is>
           <t>Phase 12 — Frontend refactor</t>
         </is>
       </c>
-      <c r="B58" s="3" t="inlineStr">
+      <c r="B59" s="3" t="inlineStr">
         <is>
           <t>DocumentEditor.tsx split (Shell/Canvas/Toolbar/useDocument/useAutoSave/useFormatting/useSelection/useHistory/useExport/usePageSettings)</t>
         </is>
       </c>
-      <c r="C58" s="4" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="D58" s="3" t="inlineStr"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="2" t="n"/>
-      <c r="B59" s="3" t="inlineStr">
-        <is>
-          <t>Server state via TanStack Query; editor state stays local</t>
-        </is>
-      </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="D59" s="3" t="inlineStr"/>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>The 500-line DocumentEditor.tsx is now editor/DocumentEditorShell.tsx, which only lays out and wires: useDocument (server state + changed-elsewhere), useAutoSave, useFormatting, useHistory (undo/redo), useSelection, useExport, usePageSettings (geometry, zoom, page count); EditorCanvas (the pages), EditorToolbar + RichTextToolbar, EditorActionBar, EditorStatusBar, EditableTitle, ExportMenu; panels/ (Templates, Instructions, PageSettings, Structure, Properties + PropertiesSidebar). EditorState.tsx gives the panels the document, editor and selection, and `change`: every change saves pending typing first -- a failed save now stops the change instead of letting it overwrite the typing (before, it went ahead). Editor components moved from components/ to editor/ with git mv. Checked live end to end.</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n"/>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>Debounced / cancelable / status-aware autosave (Saving/Saved/Failed/Offline/Conflict)</t>
+          <t>Server state via TanStack Query; editor state stays local</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="D60" s="3" t="inlineStr"/>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>@tanstack/react-query 5 (app/providers.tsx; retries only network/5xx failures). services/queries.ts: signed-in user, templates (refetched on window focus -- replaces a hand-made focus listener), a template and its versions, style previews keyed by the style (debounced; the last one stays while the next loads). The template editor keeps only unsaved edits locally; the saved template is the cache. The edited document is in the cache too (editor/useDocument.ts, seeded from the server render, gcTime 0); the Tiptap content stays local. No Redux/Zustand.</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n"/>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>Typed API client replacing ad-hoc services/api.ts fetch calls</t>
+          <t>Debounced / cancelable / status-aware autosave (Saving/Saved/Failed/Offline/Conflict)</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="D61" s="3" t="inlineStr"/>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>editor/useAutoSave.ts: one request 1.2 s after typing stops (live: 23 keystrokes, one PUT), one at a time, flush() resolves only when everything typed before it is saved. Statuses: Saving…, Saved, Failed to save (retried after 5/15/60 s or with Retry), Offline (browser offline; retried on the online event), Conflict (412: nothing more is sent, the banner offers a reload). Asks before leaving with unsaved typing; saves what is pending when the editor unmounts. Checked live: backend stopped while typing -&gt; Failed to save -&gt; saved once it was back; a write from another tab -&gt; Conflict.</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n"/>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>Editor pages like Word: separate sheets, real pagination, header/footer on every page</t>
+          <t>Typed API client replacing ad-hoc services/api.ts fetch calls</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
@@ -1593,7 +1625,7 @@
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>editor/pagination.ts: a ProseMirror plugin measures top-level blocks (and top-level list items) and inserts spacer decorations so a block that doesn't fit starts on the next page; page breaks start a new page; the real page count goes to the status bar. Each page is its own white sheet with a border and shadow on a grey desk, a gap between pages, and the header/footer/page number in each page's margins ({PAGE}/{NUMPAGES} filled in). Replaces the single white strip with faded seams (Boril asked for pages as separate boxes, as in Word or Canva). Pages shrink to fit the column until a zoom is picked. Known limit: a block taller than a page isn't split. Verified live on the stress-test document (10 Letter pages). Also seen: below ~1100 px wide the two side panels leave the editor column very narrow; worth collapsing them there.</t>
+          <t>services/api/ replaces services/api.ts: client.ts (apiFetch, ApiError with message/code/details/requestId, NetworkError, UnauthorizedError), auth, documents (write queue + revisions), jobs (typed results), templates, assets; index.ts keeps `@/services/api` imports working. Backend (корекции.docx §49): every error is {code, message, details, request_id} (app/api/errors.py), validation errors never echo input, unexpected ones are a plain 500 logged with the request id, X-Request-ID on every response (exposed to the browser). Types: types/document.ts now names the types generated from the OpenAPI schema (ApiModel base marks always-sent response fields required; job results and ApiError in the schema); the schema is a committed file from scripts/export_openapi.py, checked by tests/test_openapi_contract.py. tests/test_api_errors.py (7). 492 backend tests.</t>
         </is>
       </c>
     </row>
@@ -1601,177 +1633,213 @@
       <c r="A63" s="2" t="n"/>
       <c r="B63" s="3" t="inlineStr">
         <is>
+          <t>Editor pages like Word: separate sheets, real pagination, header/footer on every page</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>editor/pagination.ts: a ProseMirror plugin measures top-level blocks (and top-level list items) and inserts spacer decorations so a block that doesn't fit starts on the next page; page breaks start a new page; the real page count goes to the status bar. Each page is its own white sheet with a border and shadow on a grey desk, a gap between pages, and the header/footer/page number in each page's margins ({PAGE}/{NUMPAGES} filled in). Replaces the single white strip with faded seams (Boril asked for pages as separate boxes, as in Word or Canva). Pages shrink to fit the column until a zoom is picked. Known limit: a block taller than a page isn't split. Verified live on the stress-test document (10 Letter pages). Also seen: below ~1100 px wide the two side panels leave the editor column very narrow; worth collapsing them there.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n"/>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
           <t>Toolbar formatting saved with the text; real checklists</t>
         </is>
       </c>
-      <c r="C63" s="4" t="inlineStr">
-        <is>
-          <t>☑</t>
-        </is>
-      </c>
-      <c r="D63" s="3" t="inlineStr">
+      <c r="C64" s="4" t="inlineStr">
+        <is>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
         <is>
           <t>Toolbar: undo/redo, bold/italic/underline/strikethrough, super/subscript, font and size, text colour, highlight, clear formatting, alignment, bullet/numbered/check lists. Character formatting is stored as marks (textStyle font/size/colour/background, superscript, subscript) and saved by autosave; alignment outside tables is a live override like the Properties panel's. Checklists use Tiptap TaskList/TaskItem instead of a ☑/☐ text glyph (Boril: 'fix the checkboxes'), and ticking one is saved. Element ids stay stable when Enter splits a block (ids written back into the editor), and a save is skipped when nothing changed. Verified live: checkbox state, colours, highlight, superscript, line breaks and second paragraphs in table cells survive a reload.</t>
         </is>
       </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="2" t="inlineStr">
-        <is>
-          <t>Phase 13 — Dashboard &amp; document management</t>
-        </is>
-      </c>
-      <c r="B64" s="3" t="inlineStr">
-        <is>
-          <t>Post-auth dashboard (recent docs, templates, usage, quick actions)</t>
-        </is>
-      </c>
-      <c r="C64" s="4" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="D64" s="3" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n"/>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>Document list with delete wired to Phase 1's route</t>
+          <t>Side panels below ~1100 px don't crush the editor</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="D65" s="3" t="inlineStr"/>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>Below 1100 px the left flyout and the Properties sidebar open over the pages (absolute, shadowed) instead of taking their width; the toolbar gets a Properties button; the Templates panel starts closed (lib/useMediaQuery). Checked live at 740 and 1440 px.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="n"/>
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>Phase 13 — Dashboard &amp; document management</t>
+        </is>
+      </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>Document Health scoring (deterministic checks, AI only explains)</t>
+          <t>Post-auth dashboard (recent docs, templates, usage, quick actions)</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="D66" s="3" t="inlineStr"/>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>`/` signed in = components/dashboard/Dashboard.tsx (signed out: Landing): quick actions (paste, upload, match a document, templates), the 6 latest documents with status, templates with “Use” (/new?template=&lt;id&gt;; the wizard also takes ?reference=1), this month's usage (GET /api/usage) and the 5 latest exports (GET /api/jobs?type=export&amp;status=succeeded) with downloads while they last. Header gets Documents/Templates links. Checked live in Boril's account.</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n"/>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>Before/after comparison view</t>
+          <t>Document list with delete wired to Phase 1's route</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="D67" s="3" t="inlineStr"/>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>/documents (components/documents/DocumentList.tsx) on GET /api/documents: title, last change, source, status (Draft / Formatted · template name, from the new documents.formatted_at -- migration ee14c191e210 applied to Supabase, backfilled 6 of 8), search (case-insensitive, Cyrillic checked live; % and _ literal), sort (changed/created/title), 20 per page; reads a few JSON fields, never whole documents. Delete asks first (ConfirmDialog, focus on Cancel) and is permanent (§32): versions and export files go at once, images with the unused-image sweep. tests/test_document_management.py.</t>
+        </is>
+      </c>
     </row>
     <row r="68">
-      <c r="A68" s="2" t="inlineStr">
-        <is>
-          <t>Phase 14 — Billing</t>
-        </is>
-      </c>
+      <c r="A68" s="2" t="n"/>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>Entitlements service (can_export_docx, max_documents, etc. -- no scattered if plan==)</t>
+          <t>Document Health scoring (deterministic checks, AI only explains)</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="D68" s="3" t="inlineStr"/>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>formatting/health.py: 11 deterministic checks -- structure, fonts, heading sizes, spacing (+ empty paragraphs as space), direct formatting, numbering (hand-numbered gaps, doubled list numbers), alignment, tables, captions, page breaks, links (as written) -- each naming its elements; score = weighted pass (warn = half), skipped checks left out; no AI (explanations by AI left for later, never the score). GET .../health; editor Health panel with “Show” per issue. tests/test_health.py (16).</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n"/>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>Stripe integration scaffolding</t>
+          <t>Before/after comparison view</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="D69" s="3" t="inlineStr"/>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>formatting/compare.py + GET .../compare?from=&amp;to= (default original vs now): elements added/removed/moved (LCS)/retyped/edited by id; style changes per kind of text and per block formatted on its own, compared as user settings (line spacing, image alignment); page settings. /documents/{id}/compare: both versions drawn read-only by the editor's own extensions with changed blocks marked (ProseMirror decorations), the changes listed beside, version pickers, restore the “before”. tests/test_compare.py.</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n"/>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>FREE/PRO/BUSINESS plans -- NEEDS Boril's real Stripe account + pricing input</t>
+          <t>Document version history: view, restore, compare (§31)</t>
         </is>
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="D70" s="3" t="inlineStr"/>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>Versions now record what they did (DocumentVersion.description: “Applied formatting…”, “Renamed to…”, “Edited the text”, “Restored version N”); the original (version 1) is never trimmed. GET .../versions, .../versions/{n}, POST .../versions/{n}/restore (If-Match; saved as a new change, undoable). Editor History panel replaces the “Recent changes” list. Checked live: rename then restore the original.</t>
+        </is>
+      </c>
     </row>
     <row r="71">
-      <c r="A71" s="2" t="inlineStr">
-        <is>
-          <t>Phase 15 — Security hardening</t>
-        </is>
-      </c>
+      <c r="A71" s="2" t="n"/>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>Magic-byte file validation + extension allowlist + MIME check</t>
+          <t>Usage metering service (§36)</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="D71" s="3" t="inlineStr"/>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t>services/usage_service.py: a usage_records row per document created, processing job, export and completed AI call (MeteredAIProvider; a job's calls count even if it fails later), per workspace and UTC month; storage measured on request. GET /api/usage for the dashboard; Phase 14's limits will read it. Starts counting from Phase 13. tests/test_usage.py (6).</t>
+        </is>
+      </c>
     </row>
     <row r="72">
-      <c r="A72" s="2" t="n"/>
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>Phase 14 — Billing</t>
+        </is>
+      </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>Zip-bomb / decompressed-size / archive-entry-limit protection</t>
+          <t>Entitlements service (can_export_docx, max_documents, etc. -- no scattered if plan==)</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="D72" s="3" t="inlineStr"/>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>app/billing/plans.json (Free/Pro/Business: canExportDocx/Pdf, maxDocuments, maxDocumentSizeMb, maxAiOperations per UTC month, maxTemplates, maxStorageMb, priorityProcessing; null = unlimited; validated at startup) + services/entitlements_service.py: the plan from the workspace's subscriptions row (active/trialing/past_due), else Free; every check reads entitlements, never a plan name. Enforced before the work on every way in (sync endpoints, job endpoints, the job runner, DocumentService.create, AssetService.store, TemplateService.create): 402 plan_limit with entitlement/limit/used. AI: work that is all AI refused up front; optional AI steps fall back; the allowance counts the request's/job's own calls. File size capped by MAX_UPLOAD_SIZE_MB. Priority processing = arq score head start. tests/test_entitlements.py (13).</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n"/>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>Rate limiting: login, register, AI endpoints, upload, export</t>
+          <t>Stripe integration scaffolding</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="D73" s="3" t="inlineStr"/>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="inlineStr">
+        <is>
+          <t>stripe==15.6.1. billing/stripe_gateway.py (Checkout, billing portal, signature-checked events, subscription fetched fresh from Stripe) + services/billing_service.py + api/billing.py: GET /api/billing (plan, status, period end, usage vs limits, plans, billingEnabled), POST /checkout (workspace id on checkout + subscription metadata; 409 when already subscribed), POST /portal, POST /webhook (checkout.session.completed, customer.subscription.*; replays idempotent, stale news about a replaced subscription ignored). Migration 85211092fe4c (cancel_at_period_end, Stripe id indexes) applied to Supabase. Frontend /settings/billing (meters, plan cards, waits for the webhook after checkout), header card icon, dashboard plan link, a notice offering plans on any 402. tests/test_billing.py (13, real HMAC signatures).</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n"/>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>Structured audit logging with request IDs</t>
+          <t>FREE/PRO/BUSINESS plans -- NEEDS Boril's real Stripe account + pricing input</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
@@ -1779,149 +1847,355 @@
           <t>☐</t>
         </is>
       </c>
-      <c r="D74" s="3" t="inlineStr"/>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>Built with PLACEHOLDER limits and no prices (plans.json). Needs Boril: a Stripe account, a product + recurring price per paid plan, the customer portal switched on, a webhook endpoint at &lt;backend&gt;/api/billing/webhook; then STRIPE_SECRET_KEY, STRIPE_WEBHOOK_SECRET, STRIPE_PRICE_PRO, STRIPE_PRICE_BUSINESS, FRONTEND_URL in backend/.env and priceLabel per plan (README, 'Plans and billing'). Until then everyone is on Free and the billing page says paid plans aren't available.</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n"/>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>Secure headers / CORS configuration review</t>
+          <t>Plan limits in the app: billing page, limit notices (§35/§36)</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="D75" s="3" t="inlineStr"/>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>/settings/billing: current plan + status (Active/Trial/Payment overdue/Ended…), renews/ends date, usage meters (documents, AI operations this month with renewal date, templates, storage), plan cards (Upgrade → Checkout, or “Change in billing portal” when subscribed; “Not available yet” without Stripe). services/api/client.ts fires smartdoc:plan-limit on any 402 plan_limit; PlanLimitBanner offers the page. Checked live on Boril's account at 740 px and 1280 px; tsc, eslint, next build clean.</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>Phase 16 — Testing</t>
+          <t>Phase 15 — Security hardening</t>
         </is>
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>Vitest + React Testing Library set up (frontend currently has 0 tests)</t>
+          <t>Magic-byte file validation + extension allowlist + MIME check</t>
         </is>
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="D76" s="3" t="inlineStr"/>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>app/security/files.py: .docx = ZIP with [Content_Types].xml (OLE .doc/password-protected named as such), .pdf = %PDF- in the first 1 KB, .txt = no NUL bytes (UTF-16 BOM allowed); the browser's declared type must fit the extension (octet-stream = unknown); the real type replaces it before a job stores the file; 400 invalid_file before anything is queued. Inline/Word images stored only if their bytes match their type (never SVG). Instructions files too.</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n"/>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>Playwright E2E for the full workflow list (§46)</t>
+          <t>Zip-bomb / decompressed-size / archive-entry-limit protection</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="D77" s="3" t="inlineStr"/>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>check_docx before python-docx opens a package (also inside import_docx): &lt;=1000 entries, XML parts &lt;=50 MB unpacked, total &lt;=200 MB, no entry &gt;100x its packed size (from 1 MB), no absolute/.. names, no encrypted entries (zipfile never unpacks past a declared size, so declared sizes suffice). Raw XML via parse_xml_part (no entities, no DTD, no network, no huge_tree): XXE and billion-laughs tested. PDFs: &lt;=1000 pages, any pypdf error = refusal; pypdf's own 75 MB stream limits kept.</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n"/>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>Golden-document fixture suite: real DOCX upload -&gt; edit -&gt; export -&gt; re-import -&gt; compare</t>
+          <t>Rate limiting: login, register, AI endpoints, upload, export</t>
         </is>
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="D78" s="3" t="inlineStr"/>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="inlineStr">
+        <is>
+          <t>app/security/rate_limit.py: fixed windows in memory or Redis (RATE_LIMIT_BACKEND=redis; fails open with a log line). login 20/min per address + 10/min per account (hashed email), register 10/h per address, ai 20/min, upload 20/min, export 30/min per user, global 600/min per session or address (health and Stripe webhook exempt). 429 rate_limited + Retry-After; all configurable, validated at startup. tests/test_security.py.</t>
+        </is>
+      </c>
     </row>
     <row r="79">
-      <c r="A79" s="2" t="inlineStr">
-        <is>
-          <t>Phase 17 — Docker + CI/CD</t>
-        </is>
-      </c>
+      <c r="A79" s="2" t="n"/>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>Dockerfile (backend) + Dockerfile (frontend)</t>
+          <t>Structured audit logging with request IDs</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="D79" s="3" t="inlineStr"/>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="inlineStr">
+        <is>
+          <t>app/audit.py (app.audit logger) + app/logging_setup.py (text or JSON lines, request id stamped on every record, LOG_REQUESTS line per request with status/duration). Events: auth.registered/login_succeeded/login_failed (hashed email)/logout, document.created/exported/version_restored/deleted, template.created/deleted, billing.*, limit.plan_refused/rate_refused, file.refused, request.cross_site_refused. job.finished (type, outcome, duration, AI calls) and ai.call (task, duration, tokens, outcome). No content in logs: describe_error() for AI failures; tested.</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n"/>
       <c r="B80" s="3" t="inlineStr">
         <is>
-          <t>docker-compose.yml (frontend/backend/postgres/redis/minio)</t>
+          <t>Secure headers / CORS configuration review</t>
         </is>
       </c>
       <c r="C80" s="4" t="inlineStr">
         <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="D80" s="3" t="inlineStr"/>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="inlineStr">
+        <is>
+          <t>API: nosniff, X-Frame-Options DENY, Referrer-Policy no-referrer, CSP default-src 'none'; sandbox, COOP, optional HSTS (HSTS_SECONDS). Frontend (next.config.ts): CSP (self + API origin; unsafe-eval in dev only), nosniff, DENY, Permissions-Policy, no X-Powered-By. CORS: named origins only ('*' refused at startup), headers Content-Type/If-Match/X-Request-ID, Retry-After exposed. Request bodies capped (MAX_REQUEST_SIZE_MB=25) before reading. Checked live.</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n"/>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>GitHub Actions: tests/typecheck/lint/build/migration-check on PR</t>
+          <t>AI hardening: prompt separation, timeouts, telemetry, long-document chunking (§20-22)</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="D81" s="3" t="inlineStr"/>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="inlineStr">
+        <is>
+          <t>ai/prompting.py: rules in the system prompt, the document between tags with a random per-call name (can't be closed by the content; nothing in it altered). AnthropicProvider: timeout (AI_TIMEOUT_SECONDS=180), SDK retries, one ai.call log line. structure_analysis: ~8,000-char pieces cut between paragraphs, each shown the earlier headings, a failing piece falls back alone, at most 20 pieces go to the AI (the document notes the rest). Instructions list &lt;=400 elements; style analysis reads &lt;=300. tests/test_observability.py.</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n"/>
       <c r="B82" s="3" t="inlineStr">
         <is>
-          <t>Health + readiness endpoints; production ASGI (never fastapi dev in prod)</t>
+          <t>Secrets hidden, privacy messaging (§81)</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="D82" s="3" t="inlineStr"/>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="inlineStr">
+        <is>
+          <t>Anthropic/S3/Stripe secrets are SecretStr (settings print as asterisks). Landing + wizard say documents are private, the AI only reads what a task needs and never rewrites, deletion removes history; the wizard shows the plan's real file-size limit. alembic/env.py no longer disables the app's loggers when run in-process.</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
+          <t>Phase 16 — Testing</t>
+        </is>
+      </c>
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>Vitest + React Testing Library set up (frontend currently has 0 tests)</t>
+        </is>
+      </c>
+      <c r="C83" s="4" t="inlineStr">
+        <is>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="inlineStr">
+        <is>
+          <t>frontend: vitest.config.mts (jsdom), tests/setup.ts, npm test. 46 tests: the 12 golden documents (JSON from backend/scripts/export_golden_json.py, kept current by a backend test) through the real Tiptap editor and back via reconcileElements must be unchanged, and an edit changes only itself; the API client (ApiError, request ids, plan-limit event, 401 redirect, If-Match); ConfirmDialog; PlanLimitBanner; BillingPage (meters, plan cards, Checkout/portal redirects, post-checkout wait); lib/format. Found and fixed: table summary joined with tabs vs the backend's ' | ', page break inline [] vs none, footnotes saved as paragraphs (new Footnote node), a trailing blank paragraph saved after the first edit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n"/>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>Playwright E2E for the full workflow list (§46)</t>
+        </is>
+      </c>
+      <c r="C84" s="4" t="inlineStr">
+        <is>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="inlineStr">
+        <is>
+          <t>frontend/playwright.config.ts + e2e/: its own backend (backend/scripts/e2e_server.py: fresh SQLite + assets, no AI, no Stripe, no rate limits) on :8100 and a production build (.next-e2e) on :3100; Edge on Windows. 16 tests, all §46 workflows: sign up/out/in, wrong password, redirect to sign-in and back, protected document access; paste + structure review; typing autosaved and kept after reload; template choose/apply + undo/redo; DOCX + PDF export; delete; uploads with link, pictures, captions, everything; template creation; Format by Example; one approved editor screenshot (Windows). Found and fixed: header kept 'Sign in' after signing in (query cache).</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n"/>
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>Golden-document fixture suite: real DOCX upload -&gt; edit -&gt; export -&gt; re-import -&gt; compare</t>
+        </is>
+      </c>
+      <c r="C85" s="4" t="inlineStr">
+        <is>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="inlineStr">
+        <is>
+          <t>backend/tests/fixtures/documents/01-simple … 12-complex.docx (scripts/make_golden_documents.py). tests/test_golden_documents.py: per-document import assertions; import -&gt; format (academic) -&gt; DOCX export -&gt; re-import -&gt; compare every element, run, link, list level, table span/shading, picture, page setup, warnings; unformatted export keeps the source look; §45 critical round trip through the API (upload -&gt; editor-style save with an edit -&gt; format -&gt; export -&gt; re-import); SMARTDOC_REAL_DOCX runs it on any real document (Boril's stress test passes). Found and fixed: 'List Bullet 2/3' styles imported as separate flat lists; exported footnotes re-imported as paragraphs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>Phase 17 — Docker + CI/CD</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>Dockerfile (backend) + Dockerfile (frontend)</t>
+        </is>
+      </c>
+      <c r="C86" s="4" t="inlineStr">
+        <is>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="inlineStr">
+        <is>
+          <t>backend/Dockerfile: python:3.13-slim, requirements.lock with --require-hashes, Liberation + DejaVu fonts for the PDF export, non-root, uvicorn --proxy-headers (WEB_CONCURRENCY, FORWARDED_ALLOW_IPS), healthcheck; the same image runs the arq worker and `alembic upgrade head`. frontend/Dockerfile: npm ci, next build with NEXT_PUBLIC_API_BASE_URL, standalone server as node (NEXT_OUTPUT=standalone; API_INTERNAL_URL for server-side calls). Docker can't run on this machine (BIOS virtualization off): the standalone server was checked here, the images are built in CI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n"/>
+      <c r="B87" s="3" t="inlineStr">
+        <is>
+          <t>docker-compose.yml (frontend/backend/postgres/redis/minio)</t>
+        </is>
+      </c>
+      <c r="C87" s="4" t="inlineStr">
+        <is>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="inlineStr">
+        <is>
+          <t>Root docker-compose.yml: postgres:17, redis:7, MinIO + a one-shot bucket job, `migrate` (alembic upgrade head, before anything else), backend, worker (arq), frontend (API_INTERNAL_URL=http://backend:8000); healthchecks and depends_on conditions. Validated with `docker compose config`.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n"/>
+      <c r="B88" s="3" t="inlineStr">
+        <is>
+          <t>GitHub Actions: tests/typecheck/lint/build/migration-check on PR</t>
+        </is>
+      </c>
+      <c r="C88" s="4" t="inlineStr">
+        <is>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="inlineStr">
+        <is>
+          <t>.github/workflows/ci.yml on every PR and push to main: backend tests (dev lock, fonts), migrations on postgres:17 (upgrade head, alembic check, downgrade base, upgrade head), frontend lint/tsc/Vitest/build, Playwright e2e in Chromium (report kept on failure); on main only after all pass: both images built and the compose file checked. No deploy step.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n"/>
+      <c r="B89" s="3" t="inlineStr">
+        <is>
+          <t>Health + readiness endpoints; production ASGI (never fastapi dev in prod)</t>
+        </is>
+      </c>
+      <c r="C89" s="4" t="inlineStr">
+        <is>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="inlineStr">
+        <is>
+          <t>GET /api/health (liveness) and GET /api/ready (database, and Redis when jobs or rate limits use it; 503 naming the failing check), unversioned and outside the rate limits. Production ASGI: uvicorn in the image, never fastapi dev. tests/test_api_versioning.py.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n"/>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>API versioning: /api/v1 as the contract (§48)</t>
+        </is>
+      </c>
+      <c r="C90" s="4" t="inlineStr">
+        <is>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="inlineStr">
+        <is>
+          <t>All routers under /api/v1 (the only paths in the OpenAPI schema); the unversioned /api paths kept as deprecated aliases (Deprecation + Link: successor-version headers). The frontend client adds the prefix (API_PREFIX) and reads image URLs under either prefix. Tests moved to /api/v1; checked live on Boril's account.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n"/>
+      <c r="B91" s="3" t="inlineStr">
+        <is>
+          <t>Reproducible dependencies: pyproject + lockfiles (§47)</t>
+        </is>
+      </c>
+      <c r="C91" s="4" t="inlineStr">
+        <is>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="inlineStr">
+        <is>
+          <t>backend/pyproject.toml (direct deps pinned, dev extra), requirements.lock and requirements-dev.lock made by uv pip compile --universal --generate-hashes (Windows/Linux/macOS markers); requirements.txt removed. A fresh venv from the dev lock with --require-hashes passed all 643 tests. Frontend: package-lock.json + npm ci.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
           <t>Phase 18 — Final audit</t>
         </is>
       </c>
-      <c r="B83" s="3" t="inlineStr">
+      <c r="B92" s="3" t="inlineStr">
         <is>
           <t>docs/architecture/final-audit.md (A-I structure per doc §92)</t>
         </is>
       </c>
-      <c r="C83" s="4" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="D83" s="3" t="inlineStr"/>
+      <c r="C92" s="4" t="inlineStr">
+        <is>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="inlineStr">
+        <is>
+          <t>docs/architecture/final-audit.md: the §88 Definition of Done area by area and the §91 deliverables, then A-I per §92 (changed; preserved; migrations; supported, each with the tests that prove it; not supported; known limitations; tested; what to watch in production; next improvements under the §93 product rule). Written after a full re-run on 2026-09-26: 643 backend tests (+1 optional), 46 Vitest, 16 Playwright, tsc/ESLint clean; Supabase migrations and advisors checked. README status, migration-plan, target-state and current-state (marked superseded) updated, and stale README paths fixed. Open, needing Boril: Stripe account and prices; a production deployment.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="C2:C83" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C2:C92" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"☐,☑"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>